<commit_message>
Mega fix: Restored correct UI, added Logout and WhatsApp buttons, added Odometer, fixed Washing Excel, added Schedule Export, and updated Database from vehicle_lookup_v2.xlsx
</commit_message>
<xml_diff>
--- a/po_template.xlsx
+++ b/po_template.xlsx
@@ -347,7 +347,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -502,12 +502,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
@@ -1707,7 +1701,7 @@
       <c r="I3" s="5" t="n"/>
       <c r="J3" s="27" t="inlineStr">
         <is>
-          <t>NO. 000001</t>
+          <t>NO. 0144</t>
         </is>
       </c>
       <c r="K3" s="3" t="n"/>
@@ -1717,7 +1711,7 @@
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="D4" s="7" t="n"/>
@@ -1771,7 +1765,7 @@
           <t>اسم السائق:</t>
         </is>
       </c>
-      <c r="D7" s="36" t="inlineStr"/>
+      <c r="D7" s="36" t="n"/>
       <c r="E7" s="38" t="n"/>
       <c r="F7" s="9" t="inlineStr">
         <is>
@@ -1788,11 +1782,7 @@
           <t>الوظيفة:</t>
         </is>
       </c>
-      <c r="I7" s="36" t="inlineStr">
-        <is>
-          <t>سائق</t>
-        </is>
-      </c>
+      <c r="I7" s="36" t="n"/>
       <c r="J7" s="38" t="n"/>
       <c r="K7" s="3" t="n"/>
     </row>
@@ -1804,37 +1794,37 @@
           <t>نوع السيارة:</t>
         </is>
       </c>
-      <c r="D8" s="58" t="inlineStr"/>
+      <c r="D8" s="58" t="n"/>
       <c r="E8" s="38" t="n"/>
       <c r="F8" s="11" t="inlineStr">
         <is>
           <t>رقم اللوحة:</t>
         </is>
       </c>
-      <c r="G8" s="12" t="inlineStr"/>
+      <c r="G8" s="12" t="n"/>
       <c r="H8" s="11" t="inlineStr">
         <is>
           <t>الموديل:</t>
         </is>
       </c>
-      <c r="I8" s="40" t="inlineStr"/>
+      <c r="I8" s="40" t="n"/>
       <c r="J8" s="38" t="n"/>
       <c r="K8" s="3" t="n"/>
     </row>
     <row r="9" ht="18.4" customHeight="1" s="46">
       <c r="A9" s="2" t="n"/>
       <c r="B9" s="3" t="n"/>
-      <c r="C9" s="13" t="n"/>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>عداد السيارة:</t>
+        </is>
+      </c>
       <c r="D9" s="13" t="n"/>
       <c r="E9" s="13" t="n"/>
-      <c r="F9" s="62" t="inlineStr">
-        <is>
-          <t>عداد السيارة:</t>
-        </is>
-      </c>
-      <c r="G9" s="63" t="n"/>
-      <c r="H9" s="37" t="n"/>
-      <c r="I9" s="38" t="n"/>
+      <c r="F9" s="13" t="n"/>
+      <c r="G9" s="13" t="n"/>
+      <c r="H9" s="13" t="n"/>
+      <c r="I9" s="13" t="n"/>
       <c r="J9" s="13" t="n"/>
       <c r="K9" s="3" t="n"/>
     </row>
@@ -1898,13 +1888,13 @@
       <c r="C12" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="36" t="inlineStr"/>
+      <c r="D12" s="36" t="n"/>
       <c r="E12" s="37" t="n"/>
       <c r="F12" s="38" t="n"/>
       <c r="G12" s="36" t="n"/>
       <c r="H12" s="32" t="n"/>
       <c r="I12" s="32" t="n"/>
-      <c r="J12" s="36" t="inlineStr"/>
+      <c r="J12" s="36" t="n"/>
       <c r="K12" s="3" t="n"/>
     </row>
     <row r="13" ht="17.1" customHeight="1" s="46">
@@ -2002,12 +1992,12 @@
       <c r="C18" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="36" t="inlineStr"/>
+      <c r="D18" s="36" t="n"/>
       <c r="E18" s="37" t="n"/>
       <c r="F18" s="37" t="n"/>
       <c r="G18" s="38" t="n"/>
       <c r="H18" s="36" t="n"/>
-      <c r="I18" s="36" t="inlineStr"/>
+      <c r="I18" s="36" t="n"/>
       <c r="J18" s="38" t="n"/>
       <c r="K18" s="3" t="n"/>
     </row>
@@ -2124,7 +2114,7 @@
       </c>
       <c r="D24" s="36" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="E24" s="36" t="n"/>
@@ -2242,15 +2232,15 @@
       <c r="C30" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D30" s="36" t="inlineStr"/>
+      <c r="D30" s="36" t="n"/>
       <c r="E30" s="38" t="n"/>
       <c r="F30" s="36" t="n"/>
-      <c r="G30" s="36" t="inlineStr"/>
-      <c r="H30" s="36" t="inlineStr"/>
+      <c r="G30" s="36" t="n"/>
+      <c r="H30" s="36" t="n"/>
       <c r="I30" s="36" t="n"/>
       <c r="J30" s="36" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="K30" s="3" t="n"/>
@@ -2621,7 +2611,7 @@
     <row r="130" ht="18.6" customHeight="1" s="46"/>
     <row r="131" ht="18.6" customHeight="1" s="46"/>
   </sheetData>
-  <mergeCells count="40">
+  <mergeCells count="39">
     <mergeCell ref="D18:G18"/>
     <mergeCell ref="I34:J34"/>
     <mergeCell ref="D13:F13"/>
@@ -2648,7 +2638,6 @@
     <mergeCell ref="E4:H4"/>
     <mergeCell ref="E37:J37"/>
     <mergeCell ref="E38:H38"/>
-    <mergeCell ref="G9:I9"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="I17:J17"/>
     <mergeCell ref="D8:E8"/>

</xml_diff>

<commit_message>
Fix UI: Styled Odometer row in Excel template, and made all summary inputs editable in purchase.html
</commit_message>
<xml_diff>
--- a/po_template.xlsx
+++ b/po_template.xlsx
@@ -347,7 +347,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -502,6 +502,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
@@ -1814,18 +1820,18 @@
     <row r="9" ht="18.4" customHeight="1" s="46">
       <c r="A9" s="2" t="n"/>
       <c r="B9" s="3" t="n"/>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="62" t="inlineStr">
         <is>
           <t>عداد السيارة:</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n"/>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="13" t="n"/>
-      <c r="G9" s="13" t="n"/>
-      <c r="H9" s="13" t="n"/>
-      <c r="I9" s="13" t="n"/>
-      <c r="J9" s="13" t="n"/>
+      <c r="D9" s="58" t="n"/>
+      <c r="E9" s="38" t="n"/>
+      <c r="F9" s="40" t="n"/>
+      <c r="G9" s="40" t="n"/>
+      <c r="H9" s="40" t="n"/>
+      <c r="I9" s="40" t="n"/>
+      <c r="J9" s="63" t="n"/>
       <c r="K9" s="3" t="n"/>
     </row>
     <row r="10" ht="17.45" customHeight="1" s="46">
@@ -2611,7 +2617,7 @@
     <row r="130" ht="18.6" customHeight="1" s="46"/>
     <row r="131" ht="18.6" customHeight="1" s="46"/>
   </sheetData>
-  <mergeCells count="39">
+  <mergeCells count="40">
     <mergeCell ref="D18:G18"/>
     <mergeCell ref="I34:J34"/>
     <mergeCell ref="D13:F13"/>
@@ -2639,6 +2645,7 @@
     <mergeCell ref="E37:J37"/>
     <mergeCell ref="E38:H38"/>
     <mergeCell ref="I8:J8"/>
+    <mergeCell ref="D9:E9"/>
     <mergeCell ref="I17:J17"/>
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="I35:J35"/>

</xml_diff>